<commit_message>
docs(persona-18-35): move + version master action list into the focus folder
finwise-master-action-list-2026-06-28.xlsx -> docs/persona-18-35/finwise-master-action-list-v1.0-2026-06-29.xlsx
(versioned name per convention; no duplicate left in docs/). README index + generator output path updated.
</commit_message>
<xml_diff>
--- a/docs/finwise-device-test-build34.xlsx
+++ b/docs/finwise-device-test-build34.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/palakjain/Vibe_Coding/finwise/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B6B0CED-89A3-EA40-8629-56909333F242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47B850D4-BB10-3F4E-8CBD-1A04638D297C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4880" yWindow="80" windowWidth="28720" windowHeight="19880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4880" yWindow="0" windowWidth="28720" windowHeight="19880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Build 34 test" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="94">
   <si>
     <t>FinWise — Device Test · Build #34 (v1.0.8) — re-tests the 11 fixes from build #33 feedback</t>
   </si>
@@ -797,10 +797,13 @@
     <t>Result</t>
   </si>
   <si>
-    <t>Key problem still exists. Can only edit Base salary and bonus. Cannot edit - Equity Comp, Rental Property, and self- employment</t>
-  </si>
-  <si>
-    <t>Cash flow at the top should actula for the month, followed by actual for current and past months and planned for future - bar chart and table for monthly cash flow similar to one in onboarding. One should be able to click the bar for that month to have pop-up window with planned details for that month (it should use planned $$ for that month versus average)</t>
+    <t>Cash flow at the top should actual for the month, followed by actual for current and past months and planned for future - bar chart and table for monthly cash flow similar to one in onboarding. One should be able to click the bar for that month to have pop-up window with planned details for that month (it should use planned $$ for that month versus average)</t>
+  </si>
+  <si>
+    <t>Keyboard problem still exists. Can only edit Base salary and bonus. Cannot edit - Equity Comp, Rental Property, and self- employment</t>
+  </si>
+  <si>
+    <t>$6908 funded this month still showing behind why?</t>
   </si>
 </sst>
 </file>
@@ -856,19 +859,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1671,52 +1670,52 @@
         <v>69</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="F28" s="1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="F29" s="1" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="F30" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="F31" s="1" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="F32" s="1" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="33" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="6:6" ht="17" x14ac:dyDescent="0.2">
       <c r="F33" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="36" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="6:6" ht="34" x14ac:dyDescent="0.2">
       <c r="F36" s="1" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="37" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="6:6" ht="17" x14ac:dyDescent="0.2">
       <c r="F37" s="1" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="38" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="6:6" ht="34" x14ac:dyDescent="0.2">
       <c r="F38" s="1" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="39" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="6:6" ht="51" x14ac:dyDescent="0.2">
       <c r="F39" s="1" t="s">
         <v>79</v>
       </c>
@@ -1734,86 +1733,88 @@
   <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="139.83203125" style="5" customWidth="1"/>
-    <col min="2" max="2" width="17.5" style="2" customWidth="1"/>
-    <col min="3" max="3" width="21.33203125" style="2" customWidth="1"/>
-    <col min="4" max="16384" width="10.83203125" style="2"/>
+    <col min="1" max="1" width="139.83203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5" customWidth="1"/>
+    <col min="3" max="3" width="21.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>90</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="36" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s">
         <v>60</v>
       </c>
+      <c r="C2" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="3" spans="1:3" ht="36" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="36" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="36" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="36" x14ac:dyDescent="0.2">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="36" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" t="s">
         <v>58</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="36" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C8" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="36" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>91</v>
-      </c>
-    </row>
     <row r="9" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="18" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>89</v>
       </c>
     </row>

</xml_diff>